<commit_message>
Cambios de latam, europa y asia
</commit_message>
<xml_diff>
--- a/storage/app/pdfs/perfiles_descarga.xlsx
+++ b/storage/app/pdfs/perfiles_descarga.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://faro90mx-my.sharepoint.com/personal/rfavela_hcx_mx/Documents/F90/Operacion/Proyectos/Proyectos en curso/US Grains_007 (online tool update)/Entregable/1. Profiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://faro90mx-my.sharepoint.com/personal/rfavela_hcx_mx/Documents/F90/Operacion/Proyectos/Proyectos en curso/US Grains 013 (Analisis Global)/Latinoamerica/6.  Informacion Latam/1. Profiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="690" documentId="8_{7FF05819-4066-4415-890C-204B528D78D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D24C117D-6D7A-F645-9AB0-F10D1ABC9B5F}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{86CA14A3-0423-6B41-9947-552376DEE6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DB27E61-2420-9449-81E7-D1BA60A2D23B}"/>
   <bookViews>
-    <workbookView xWindow="2980" yWindow="4180" windowWidth="20960" windowHeight="9740" firstSheet="7" activeTab="13" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
+    <workbookView xWindow="3360" yWindow="6300" windowWidth="20960" windowHeight="9740" activeTab="4" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
   </bookViews>
   <sheets>
     <sheet name="Contenido" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="Perú" sheetId="20" r:id="rId16"/>
     <sheet name="Uruguay" sheetId="21" r:id="rId17"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" iterate="1" iterateDelta="1.0000000000000001E-5"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -754,12 +754,6 @@
     <t>&lt; 0,25 mg/l</t>
   </si>
   <si>
-    <t>Resolución 576/2019</t>
-  </si>
-  <si>
-    <t>Resolución 40103 de 2021</t>
-  </si>
-  <si>
     <t>Gasolina Corriente</t>
   </si>
   <si>
@@ -824,6 +818,12 @@
   </si>
   <si>
     <t>&lt; 3,45 %m/m</t>
+  </si>
+  <si>
+    <t>Resolución576/2019 y Resolución 492/2023</t>
+  </si>
+  <si>
+    <t>Resolución 40444 de 2023</t>
   </si>
 </sst>
 </file>
@@ -1204,14 +1204,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1249,7 +1245,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1355,7 +1351,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1497,7 +1493,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4617,16 +4613,16 @@
         <v>35</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F8" s="11" t="s">
         <v>36</v>
@@ -4646,16 +4642,16 @@
         <v>37</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>39</v>
@@ -4675,16 +4671,16 @@
         <v>40</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="F10" s="11" t="s">
         <v>42</v>
@@ -4868,10 +4864,10 @@
         <v>231</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F17" s="11" t="s">
         <v>63</v>
@@ -5606,7 +5602,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="C4" s="29"/>
       <c r="D4" s="29"/>
@@ -6806,16 +6802,16 @@
         <v>20</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F4" s="29" t="s">
         <v>21</v>
@@ -6852,10 +6848,10 @@
         <v>23</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>179</v>
@@ -6875,16 +6871,16 @@
         <v>28</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>31</v>
@@ -7359,7 +7355,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>234</v>
+        <v>256</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="31"/>
@@ -7376,7 +7372,7 @@
         <v>22</v>
       </c>
       <c r="B5" s="30">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C5" s="31"/>
       <c r="D5" s="31"/>
@@ -7416,16 +7412,16 @@
         <v>28</v>
       </c>
       <c r="B7" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="E7" s="16" t="s">
         <v>236</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>237</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>238</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>31</v>
@@ -7445,10 +7441,10 @@
         <v>35</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>112</v>
@@ -7474,7 +7470,7 @@
         <v>37</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>39</v>
@@ -7648,7 +7644,7 @@
         <v>57</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>126</v>
@@ -7657,7 +7653,7 @@
         <v>116</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="11"/>
@@ -8332,7 +8328,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C4" s="35"/>
       <c r="D4" s="35"/>
@@ -8534,16 +8530,16 @@
         <v>45</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>47</v>
@@ -8592,7 +8588,7 @@
         <v>53</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C14" s="14" t="s">
         <v>212</v>
@@ -8665,10 +8661,10 @@
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F17" s="11" t="s">
         <v>63</v>

</xml_diff>